<commit_message>
Add maximized live run shortcut and recorded DGX workbook updates
</commit_message>
<xml_diff>
--- a/excels/dgx_demo_complete_example_cn.xlsx
+++ b/excels/dgx_demo_complete_example_cn.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Y7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1303,6 +1303,352 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>创建新的 DGX exercise 并进入 Site Conf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>exercise 创建</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>dgx,demo,recorded,create</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>DGX 管理页可正常访问，并允许创建新的 exercise。</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>DATA_DGX_RECORDED_02</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>chromium</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>case_retry_1</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>能够成功创建新的 DGX exercise，并进入对应的 Site Conf 页面。</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>exercise 名称来自 Test_Data.project_name；创建后路由是动态生成的，因此只断言 /dgx/* 路由模式。</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>基于 2026-03-24 的真实录制整理，保留稳定的创建与进场链路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>完成 Site Conf 并进入 Surrounding Conf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Site Conf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>dgx,demo,recorded,siteconf</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>已经创建好新的 exercise，且浏览器已位于该 exercise 的 Site Conf 页面。</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>DATA_DGX_RECORDED_02</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>chromium</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>case_retry_1</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>能够完成 Set Boundaries 和数值输入，并进入 Surrounding Conf。</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>录制流程中共有 8 个图层下拉框被设为 Not Required；两个数值输入保留录制时的 35 和 1。</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>依赖 DGX_004，并在同一个浏览器页面连续执行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>浏览 Surrounding Conf 中的 POI 和 Land Cover 表单</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Surrounding Conf</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>dgx,demo,recorded,surrounding</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>已完成 Site Conf，浏览器位于 Surrounding Conf 的 Buildings 视图。</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>DATA_DGX_RECORDED_02</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>chromium</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>case_retry_1</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>能够打开并关闭 building 详情、POI 表单和 Land Cover 表单。</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>录制里还包含地图绘制和文件上传探索；当前用例优先保留执行器已稳定支持的部分。</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>地图多点绘制和文件上传相关控件已补入对象库，后续可继续扩展自动化能力。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="anysvml"/>
@@ -1315,7 +1661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4052,6 +4398,3937 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>打开 DGX 管理页</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>open_page</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>DGXManagePage</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>dom_ready</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Enter the DGX home page as the starting point of the recorded flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>断言已进入 DGX 首页</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>assert_url_contains</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>DGXManagePage</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://dgx.xlook.ai/</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>The URL should stay under the DGX root site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>点击 Create New DGX Exercise</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>DGXManagePage</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>create_exercise_button</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Create exercise button</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Open the dialog for creating a new exercise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>输入新的 exercise 名称</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>input_text</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DGXManagePage</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>exercise_name_input</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>${project_name}</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Exercise name input</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Use the exercise name stored in Test_Data.project_name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>提交 exercise 创建</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DGXManagePage</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>create_exercise_submit_button</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Create dialog submit button</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Submit the new exercise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>等待进入新的 exercise 路由</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>wait_url</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://dgx.xlook.ai/dgx/*</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>load</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>The newly created exercise should navigate to a dynamic /dgx/* route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>7</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>断言页面标题显示新的 exercise 名称</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>assert_text_equals</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>exercise_title_heading</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>${project_name}</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Exercise title heading</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>The page title should match the exercise name that was just created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>点击 plot 标记点</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>plot_marker_button</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Plot marker</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Open the plot popover on the map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>断言 Go to Configuration 可见</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>plot_go_to_configuration_button</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Go to Configuration button</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>The plot popover should expose the configuration entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>10</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>点击 Go to Configuration</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>plot_go_to_configuration_button</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Go to Configuration button</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Enter the Site Conf workspace for the selected plot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DGX_004</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>11</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>断言 Set Boundaries 可见</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>set_boundaries_button</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Set Boundaries entry</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>The Site Conf page should expose the Set Boundaries entry point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>点击 Set Boundaries</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>set_boundaries_button</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Set Boundaries entry</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Open the boundary configuration flow inside Site Conf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>点击 UploadPlot CAD File</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>upload_plot_button</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>UploadPlot CAD File button</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Open the layer selection modal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>断言第一个图层选择器可见</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>layer_select_button_1</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Layer selector 1</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>The first layer selector should appear after the modal opens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>打开图层选择器 1</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>layer_select_button_1</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Layer selector 1</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Open the first layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>将图层 1 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Set layer 1 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>打开图层选择器 2</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>layer_select_button_2</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Layer selector 2</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Open the second layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>7</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>将图层 2 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Set layer 2 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>打开图层选择器 3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>layer_select_button_3</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Layer selector 3</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Open the third layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>9</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>将图层 3 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Set layer 3 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>10</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>打开图层选择器 4</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>layer_select_button_4</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P57" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Layer selector 4</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Open the fourth layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>11</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>将图层 4 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P58" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Set layer 4 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>12</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>打开图层选择器 5</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>layer_select_button_5</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P59" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Layer selector 5</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Open the fifth layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>13</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>将图层 5 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Set layer 5 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>14</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>打开图层选择器 6</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>layer_select_button_6</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P61" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Layer selector 6</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Open the sixth layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>15</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>将图层 6 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P62" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Set layer 6 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>16</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>打开图层选择器 7</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>layer_select_button_7</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P63" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Layer selector 7</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Open the seventh layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>17</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>将图层 7 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Set layer 7 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>18</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>打开图层选择器 8</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>layer_select_button_8</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P65" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Layer selector 8</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Open the eighth layer selector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>19</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>将图层 8 设置为 Not Required</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>not_required_option</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P66" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Not Required option</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Set layer 8 to Not Required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>20</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>保存边界弹窗配置</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>boundary_modal_save_button</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P67" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Boundary modal save button</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Save the current layer settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>21</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>断言边界弹窗已关闭</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>assert_element_hidden</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>layer_select_button_1</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="P68" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Layer selector 1</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>The layer selector should disappear once the modal is saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>22</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>点击 Next 进入下一配置步骤</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>next_button</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P69" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Site Conf Next button</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Move to the next Site Conf step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>23</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>再次点击 Next 进入数值输入步骤</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>next_button</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P70" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Site Conf Next button</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Move to the step that contains the two numeric inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>24</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>填写第一个数值输入框为 35</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>clear_and_input</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>plot_assignment_input_1</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P71" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Numeric input 1</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>The first numeric input in the recording was set to 35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>25</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>填写第二个数值输入框为 1</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>clear_and_input</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>plot_assignment_input_2</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P72" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Numeric input 2</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>The second numeric input in the recording was set to 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>26</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>点击 Done 完成 Site Conf</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>DGXRecordedSiteConfPage</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>done_button</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P73" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Site Conf Done button</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Finish Site Conf and move into Surrounding Conf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DGX_005</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>27</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>断言 Surrounding Next 按钮可见</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>surrounding_next_button</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P74" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Surrounding Next button</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>The flow should now be inside Surrounding Conf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>打开第一条 Buildings 记录</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>surrounding_building_row_1</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P75" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>First Buildings row</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Open the detail popup of the first building row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>断言 building 详情关闭按钮可见</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>building_detail_close_button</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P76" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Building detail close button</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>The detail popup should appear after clicking the row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>关闭 building 详情浮层</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>building_detail_close_button</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P77" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Building detail close button</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Return to the Buildings list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>点击 Next 进入 POI 视图</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>surrounding_next_button</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P78" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Surrounding Next button</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Move from Buildings to POI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>断言 Add Custom POI 按钮可见</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>add_custom_poi_button</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P79" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Add Custom POI button</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>The POI view should allow opening the custom POI form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>打开自定义 POI 表单</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>add_custom_poi_button</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P80" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Add Custom POI button</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Open the POI form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>7</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>断言 POI 名称输入框可见</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>poi_name_input</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P81" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>POI name input</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>The POI form should expose the name input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>8</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>点击 Cancel 关闭 POI 表单</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>poi_cancel_button</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P82" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>POI cancel button</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Close the POI form and return to the list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>9</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>断言已返回 POI 列表</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>add_custom_poi_button</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P83" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Add Custom POI button</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>The Add Custom POI button should be visible again after canceling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>10</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>点击 Next 进入 Roads 视图</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>surrounding_next_button</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P84" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Surrounding Next button</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Move from POI to Roads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>11</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>点击 Next 进入 Land Cover 视图</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>surrounding_next_button</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P85" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Surrounding Next button</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Move from Roads to Land Cover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>12</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>断言 Add Custom Land Cover 按钮可见</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>add_custom_land_cover_button</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P86" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Add Custom Land Cover button</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>The Land Cover view should allow opening the custom form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>13</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>打开自定义 Land Cover 表单</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>add_custom_land_cover_button</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P87" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Add Custom Land Cover button</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Open the Land Cover form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>14</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>断言 Land Cover 名称输入框可见</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>land_cover_name_input</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P88" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Land Cover name input</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>The Land Cover form should expose the name input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>15</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>填写自定义 Land Cover 名称</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>input_text</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>land_cover_name_input</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>${project_result_name}</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P89" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Land Cover name input</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Use Test_Data.project_result_name as the custom Land Cover name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>16</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>选择 Land Cover 类型为 plaza</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>select_option</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>land_cover_type_select</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>plaza</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P90" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Land Cover type select</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>The recorded flow ended on the plaza option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>17</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>断言 Start Draw 按钮可见</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>land_cover_start_draw_button</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P91" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Land Cover Start Draw button</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>The form should be ready to enter draw mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>18</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>点击 Cancel 关闭 Land Cover 表单</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>land_cover_cancel_button</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P92" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Land Cover cancel button</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Close the Land Cover form. The multi-point map draw remains for a later executor enhancement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DGX_006</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>19</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>断言 Land Cover 页面仍可见 Done</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>DGXRecordedSurroundingPage</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>surrounding_done_button</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P93" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Surrounding Done button</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>After closing the form, the page should still expose the final Done button.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="anysvml"/>
@@ -4064,7 +8341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -4166,6 +8443,48 @@
       <c r="H2" s="1" t="inlineStr">
         <is>
           <t>这组数据用于驱动当前 DGX Demo 完整示例；若项目名称变化，可先在这里修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DATA_DGX_RECORDED_02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DGX 录制流程数据</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>自动化流程测试 2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>测试地表覆盖名称</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>project_name 用作 exercise 名称，project_result_name 用作自定义 land cover 名称；数值 35 和 1 保留在步骤 value 中。</t>
         </is>
       </c>
     </row>

</xml_diff>